<commit_message>
Add dahsboard preview to README
</commit_message>
<xml_diff>
--- a/results/Automobile_Insurance_Pricing_Analysis.xlsx
+++ b/results/Automobile_Insurance_Pricing_Analysis.xlsx
@@ -1309,13 +1309,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>571500</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
       <xdr:row>34</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1369,13 +1369,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>571500</xdr:colOff>
       <xdr:row>35</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
       <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>

</xml_diff>